<commit_message>
fix(excel): overwrite master excel files directly with exact github dashboard win rates and clean up temp versions
</commit_message>
<xml_diff>
--- a/final_report/GitHub_Dashboard_17_Quarters_Master.xlsx
+++ b/final_report/GitHub_Dashboard_17_Quarters_Master.xlsx
@@ -581,7 +581,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -1369,7 +1369,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -5214,7 +5214,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -9059,7 +9059,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -12904,7 +12904,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -16749,7 +16749,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -20594,7 +20594,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -24439,7 +24439,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -28284,7 +28284,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -32129,7 +32129,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -35974,7 +35974,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -39819,7 +39819,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -43664,7 +43664,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -47509,7 +47509,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -51354,7 +51354,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -55199,7 +55199,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -59044,7 +59044,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -62889,7 +62889,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>

</xml_diff>